<commit_message>
Correct seven points in Modes of Data Collection
The five workbooks are realistic teaching data, and their Notes sheets now say so. The scraping workbook cites the sampling chapters as 63 and 64 and survey design as 69, and the observation workbook's observer IDs now agree with each session's method. The sensor stream reads one machine per minute across the line, media-bias raters are described as they work, much of machine learning's raw input is found data, and the survey case study closes the part.
</commit_message>
<xml_diff>
--- a/chapters/collection/clickstream_logs.xlsx
+++ b/chapters/collection/clickstream_logs.xlsx
@@ -1900,7 +1900,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Notes for the analyst</t>
+          <t>Notes for the analyst (a realistic teaching dataset written for the book)</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>One row per event; you only capture events you INSTRUMENTED — untagged actions are invisible (missing by design).</t>
+          <t>One row per event; you only capture events you INSTRUMENTED, and untagged actions are invisible (missing by design).</t>
         </is>
       </c>
     </row>
@@ -1928,7 +1928,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Clean before analysis: drop is_bot=1, and remember this is NOT a designed sample — it reflects whoever used the product.</t>
+          <t>Clean before analysis: drop is_bot=1, and remember this is NOT a designed sample, since it reflects whoever used the product.</t>
         </is>
       </c>
     </row>

</xml_diff>